<commit_message>
Remove a menção a dados de exemplo da planilha
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KGJDSpgCByawVvtLiFnrss
</commit_message>
<xml_diff>
--- a/criterio_brasil.xlsx
+++ b/criterio_brasil.xlsx
@@ -28,7 +28,7 @@
     <t xml:space="preserve">Critério Brasil · compradores do Trident Fresh Wave</t>
   </si>
   <si>
-    <t xml:space="preserve">40 pessoas que comprariam com certeza ou provavelmente · dados de exemplo</t>
+    <t xml:space="preserve">40 pessoas que comprariam com certeza ou provavelmente</t>
   </si>
   <si>
     <t xml:space="preserve">Classe</t>
@@ -217,7 +217,7 @@
     <t xml:space="preserve">Pontos até</t>
   </si>
   <si>
-    <t xml:space="preserve">Fonte: ABEP, Critério de Classificação Econômica Brasil 2022. Dados de exemplo.</t>
+    <t xml:space="preserve">Fonte: ABEP, Critério de Classificação Econômica Brasil 2022.</t>
   </si>
   <si>
     <t xml:space="preserve">Instrução</t>
@@ -887,11 +887,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="60971539"/>
-        <c:axId val="89309913"/>
+        <c:axId val="453034"/>
+        <c:axId val="19268766"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60971539"/>
+        <c:axId val="453034"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -923,7 +923,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="89309913"/>
+        <c:crossAx val="19268766"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -931,7 +931,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="89309913"/>
+        <c:axId val="19268766"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -963,7 +963,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60971539"/>
+        <c:crossAx val="453034"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1002,9 +1002,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>387360</xdr:colOff>
+      <xdr:colOff>387000</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>32400</xdr:rowOff>
+      <xdr:rowOff>32040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1013,7 +1013,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="0" y="3695760"/>
-        <a:ext cx="5039280" cy="2699280"/>
+        <a:ext cx="5038920" cy="2698920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1424,14 +1424,14 @@
   <dimension ref="A1:T41"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="6" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="17" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="6" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="17" style="1" width="17"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>